<commit_message>
feat(battlepass): a pass lasts a Volume, not a week
The simulator finished the pass on day 7 at 20 minutes a day and day 3 at
an hour: 28,420 XP was a week's play. Tiers now cost 1,200 XP for the first
and 80 more for each after, 152,880 in all, which the simulator finishes on
day 34 at 20 minutes a day of duels, day 41 at 20 minutes a day alone and
day 15 at an hour a day; the Trials farmer never does. tests/Pacing.spec.luau
holds the 20-minute profiles between day 28 and day 42 and the hour after
day 14, and BattlepassConfig, GAME_DESIGN and ECONOMY quote those days
rather than an estimate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/economy/Vellum-economie.xlsx
+++ b/docs/economy/Vellum-economie.xlsx
@@ -791,16 +791,16 @@
         <v>5258</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2050</v>
+        <v>700</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>850</v>
+        <v>100</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -822,16 +822,16 @@
         <v>10567</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4255</v>
+        <v>1405</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>655</v>
+        <v>205</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -853,16 +853,16 @@
         <v>15025</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>5995</v>
+        <v>1975</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>1795</v>
+        <v>175</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -884,16 +884,16 @@
         <v>19533</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>8080</v>
+        <v>2340</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>2080</v>
+        <v>540</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -915,16 +915,16 @@
         <v>24091</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>10000</v>
+        <v>3000</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>2200</v>
+        <v>600</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -946,16 +946,16 @@
         <v>28750</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>13140</v>
+        <v>3750</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>3540</v>
+        <v>1350</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -977,16 +977,16 @@
         <v>33608</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>16380</v>
+        <v>4460</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>2780</v>
+        <v>260</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -1008,16 +1008,16 @@
         <v>39766</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>18320</v>
+        <v>5520</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>720</v>
+        <v>1320</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -1039,16 +1039,16 @@
         <v>44174</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>18635</v>
+        <v>6035</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1035</v>
+        <v>35</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -1070,16 +1070,16 @@
         <v>48633</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>18975</v>
+        <v>6375</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>1375</v>
+        <v>375</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -1101,16 +1101,16 @@
         <v>53141</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>19340</v>
+        <v>6960</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>1740</v>
+        <v>960</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -1132,16 +1132,16 @@
         <v>57699</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>19730</v>
+        <v>7850</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>2130</v>
+        <v>50</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -1163,16 +1163,16 @@
         <v>62358</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>20170</v>
+        <v>8570</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>2570</v>
+        <v>770</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15">
@@ -1194,16 +1194,16 @@
         <v>67216</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>20710</v>
+        <v>9110</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>3110</v>
+        <v>1310</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
@@ -1225,16 +1225,16 @@
         <v>73374</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>21400</v>
+        <v>10420</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>3800</v>
+        <v>2620</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -1256,16 +1256,16 @@
         <v>77782</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>21715</v>
+        <v>11075</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>4115</v>
+        <v>3275</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18">
@@ -1287,16 +1287,16 @@
         <v>82241</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>22055</v>
+        <v>11775</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>455</v>
+        <v>3975</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19">
@@ -1318,16 +1318,16 @@
         <v>86749</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>22420</v>
+        <v>12140</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>820</v>
+        <v>340</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20">
@@ -1349,16 +1349,16 @@
         <v>91307</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>22810</v>
+        <v>12910</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>1210</v>
+        <v>1110</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21">
@@ -1380,16 +1380,16 @@
         <v>95965</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>23250</v>
+        <v>13750</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>1650</v>
+        <v>1950</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22">
@@ -1411,16 +1411,16 @@
         <v>100824</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>23790</v>
+        <v>14710</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>2190</v>
+        <v>1110</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23">
@@ -1442,16 +1442,16 @@
         <v>106082</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>24280</v>
+        <v>15640</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>2680</v>
+        <v>2040</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24">
@@ -1473,16 +1473,16 @@
         <v>111390</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>24795</v>
+        <v>16155</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>3195</v>
+        <v>2555</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25">
@@ -1504,16 +1504,16 @@
         <v>115849</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>25135</v>
+        <v>16955</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>3535</v>
+        <v>3355</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26">
@@ -1535,16 +1535,16 @@
         <v>120357</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>25500</v>
+        <v>17800</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>3900</v>
+        <v>4200</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27">
@@ -1566,16 +1566,16 @@
         <v>124915</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>25890</v>
+        <v>18690</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>4290</v>
+        <v>1090</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28">
@@ -1597,16 +1597,16 @@
         <v>129573</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>26330</v>
+        <v>19680</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>4730</v>
+        <v>2080</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29">
@@ -1628,16 +1628,16 @@
         <v>134432</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>26870</v>
+        <v>20220</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>5270</v>
+        <v>2620</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30">
@@ -1659,16 +1659,16 @@
         <v>139690</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>27360</v>
+        <v>20710</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>5760</v>
+        <v>3110</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31">
@@ -1690,16 +1690,16 @@
         <v>144998</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>27875</v>
+        <v>21825</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>6275</v>
+        <v>4225</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32">
@@ -1721,16 +1721,16 @@
         <v>149456</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>28215</v>
+        <v>22815</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>6615</v>
+        <v>1215</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33">
@@ -1752,16 +1752,16 @@
         <v>153965</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>28580</v>
+        <v>23880</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>6980</v>
+        <v>2280</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="34">
@@ -1783,16 +1783,16 @@
         <v>158523</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>28970</v>
+        <v>25020</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>7370</v>
+        <v>3420</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="35">
@@ -1814,16 +1814,16 @@
         <v>163181</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>29410</v>
+        <v>25460</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>7810</v>
+        <v>3860</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="36">
@@ -1845,16 +1845,16 @@
         <v>168040</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>29950</v>
+        <v>26000</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>350</v>
+        <v>4400</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37">
@@ -1876,16 +1876,16 @@
         <v>173298</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>30440</v>
+        <v>27290</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>840</v>
+        <v>5690</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38">
@@ -1907,16 +1907,16 @@
         <v>178606</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>30955</v>
+        <v>28705</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>1355</v>
+        <v>7105</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39">
@@ -1938,16 +1938,16 @@
         <v>183064</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>31295</v>
+        <v>30045</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>1695</v>
+        <v>445</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40">
@@ -1969,16 +1969,16 @@
         <v>187573</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>31660</v>
+        <v>30410</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>2060</v>
+        <v>810</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="41">
@@ -2000,7 +2000,7 @@
         <v>192131</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>32050</v>
@@ -2009,7 +2009,7 @@
         <v>2450</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="42">
@@ -2409,10 +2409,10 @@
         <v>37820</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>8220</v>
+        <v>220</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55">
@@ -2440,10 +2440,10 @@
         <v>38210</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>8610</v>
+        <v>610</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="56">
@@ -2651,16 +2651,16 @@
         <v>4246</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>2220</v>
+        <v>870</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>1020</v>
+        <v>270</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -2682,16 +2682,16 @@
         <v>9191</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>5065</v>
+        <v>1895</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>1465</v>
+        <v>695</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64">
@@ -2713,16 +2713,16 @@
         <v>13287</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>7625</v>
+        <v>2785</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>1625</v>
+        <v>985</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -2744,16 +2744,16 @@
         <v>18582</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>10990</v>
+        <v>3990</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>990</v>
+        <v>1590</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66">
@@ -2775,16 +2775,16 @@
         <v>22778</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>14400</v>
+        <v>5010</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>2600</v>
+        <v>810</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="67">
@@ -2806,16 +2806,16 @@
         <v>26823</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>17810</v>
+        <v>5890</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>210</v>
+        <v>1690</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
     </row>
     <row r="68">
@@ -2837,16 +2837,16 @@
         <v>31569</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>19970</v>
+        <v>7170</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>2370</v>
+        <v>1170</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="69">
@@ -2868,16 +2868,16 @@
         <v>35564</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>20580</v>
+        <v>7980</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>2980</v>
+        <v>1980</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="70">
@@ -2899,16 +2899,16 @@
         <v>40510</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>21415</v>
+        <v>9035</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>3815</v>
+        <v>1235</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="71">
@@ -2930,16 +2930,16 @@
         <v>44605</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>22075</v>
+        <v>9935</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>475</v>
+        <v>2135</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="72">
@@ -2961,16 +2961,16 @@
         <v>49651</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>22960</v>
+        <v>11360</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>1360</v>
+        <v>1760</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
     <row r="73">
@@ -2992,16 +2992,16 @@
         <v>53847</v>
       </c>
       <c r="F73" s="2" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>23670</v>
+        <v>12070</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>2070</v>
+        <v>2470</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="74">
@@ -3023,16 +3023,16 @@
         <v>58142</v>
       </c>
       <c r="F74" s="2" t="n">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>24430</v>
+        <v>13450</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>2830</v>
+        <v>3850</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="75">
@@ -3054,16 +3054,16 @@
         <v>62888</v>
       </c>
       <c r="F75" s="2" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="G75" s="2" t="n">
-        <v>25340</v>
+        <v>14700</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>3740</v>
+        <v>1100</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="76">
@@ -3085,16 +3085,16 @@
         <v>68033</v>
       </c>
       <c r="F76" s="2" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>26200</v>
+        <v>15920</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>4600</v>
+        <v>2320</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="77">
@@ -3116,16 +3116,16 @@
         <v>72979</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>27035</v>
+        <v>17135</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>5435</v>
+        <v>3535</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="78">
@@ -3147,16 +3147,16 @@
         <v>77324</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>27745</v>
+        <v>18245</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>6145</v>
+        <v>645</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="79">
@@ -3178,16 +3178,16 @@
         <v>82370</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>28630</v>
+        <v>19990</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>7030</v>
+        <v>2390</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="80">
@@ -3209,16 +3209,16 @@
         <v>86815</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>29390</v>
+        <v>20750</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>7790</v>
+        <v>3150</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="81">
@@ -3240,16 +3240,16 @@
         <v>91111</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>30150</v>
+        <v>21970</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>550</v>
+        <v>4370</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="82">
@@ -3271,16 +3271,16 @@
         <v>95356</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>30960</v>
+        <v>23260</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>1360</v>
+        <v>5660</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="83">
@@ -3302,16 +3302,16 @@
         <v>99602</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>31620</v>
+        <v>24420</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>2020</v>
+        <v>6820</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="84">
@@ -3333,16 +3333,16 @@
         <v>104548</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>32455</v>
+        <v>25805</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>2855</v>
+        <v>4205</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="85">
@@ -3364,16 +3364,16 @@
         <v>108643</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>33115</v>
+        <v>26465</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>3515</v>
+        <v>4865</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="86">
@@ -3395,16 +3395,16 @@
         <v>113939</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>34050</v>
+        <v>28000</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>4450</v>
+        <v>6400</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="87">
@@ -3426,16 +3426,16 @@
         <v>118384</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>34810</v>
+        <v>29410</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>5210</v>
+        <v>7810</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="88">
@@ -3457,16 +3457,16 @@
         <v>122680</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>35570</v>
+        <v>30870</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>5970</v>
+        <v>1270</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="89">
@@ -3488,16 +3488,16 @@
         <v>127425</v>
       </c>
       <c r="F89" s="2" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>36480</v>
+        <v>32530</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>6880</v>
+        <v>2930</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="90">
@@ -3519,16 +3519,16 @@
         <v>131421</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>37090</v>
+        <v>33140</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>7490</v>
+        <v>3540</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="91">
@@ -3550,16 +3550,16 @@
         <v>136616</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>37975</v>
+        <v>34825</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>375</v>
+        <v>5225</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="92">
@@ -3581,16 +3581,16 @@
         <v>140712</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>38635</v>
+        <v>36385</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>1035</v>
+        <v>6785</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="93">
@@ -3612,16 +3612,16 @@
         <v>146008</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>39570</v>
+        <v>38320</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>1970</v>
+        <v>720</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="94">
@@ -3643,7 +3643,7 @@
         <v>150453</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G94" s="2" t="n">
         <v>40330</v>
@@ -3652,7 +3652,7 @@
         <v>2730</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="95">
@@ -3866,10 +3866,10 @@
         <v>45900</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>300</v>
+        <v>8300</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="102">
@@ -4511,16 +4511,16 @@
         <v>10817</v>
       </c>
       <c r="F122" s="2" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>5835</v>
+        <v>2075</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>1035</v>
+        <v>875</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="123">
@@ -4542,16 +4542,16 @@
         <v>21683</v>
       </c>
       <c r="F123" s="2" t="n">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>13005</v>
+        <v>4205</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>1805</v>
+        <v>605</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="124">
@@ -4573,16 +4573,16 @@
         <v>31700</v>
       </c>
       <c r="F124" s="2" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="G124" s="2" t="n">
-        <v>19120</v>
+        <v>6320</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>7320</v>
+        <v>320</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="125">
@@ -4604,16 +4604,16 @@
         <v>41767</v>
       </c>
       <c r="F125" s="2" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="G125" s="2" t="n">
-        <v>20560</v>
+        <v>8180</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>4760</v>
+        <v>2180</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="126">
@@ -4635,16 +4635,16 @@
         <v>51883</v>
       </c>
       <c r="F126" s="2" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G126" s="2" t="n">
-        <v>22025</v>
+        <v>10425</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>6225</v>
+        <v>2625</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="127">
@@ -4666,16 +4666,16 @@
         <v>61850</v>
       </c>
       <c r="F127" s="2" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="G127" s="2" t="n">
-        <v>23490</v>
+        <v>12850</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>5890</v>
+        <v>3250</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="128">
@@ -4697,16 +4697,16 @@
         <v>72266</v>
       </c>
       <c r="F128" s="2" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="G128" s="2" t="n">
-        <v>25105</v>
+        <v>15205</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>3505</v>
+        <v>1605</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="129">
@@ -4728,16 +4728,16 @@
         <v>83083</v>
       </c>
       <c r="F129" s="2" t="n">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="G129" s="2" t="n">
-        <v>26670</v>
+        <v>18030</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>5070</v>
+        <v>430</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="130">
@@ -4759,16 +4759,16 @@
         <v>93950</v>
       </c>
       <c r="F130" s="2" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="G130" s="2" t="n">
-        <v>28260</v>
+        <v>20560</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>6660</v>
+        <v>2960</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="131">
@@ -4790,16 +4790,16 @@
         <v>104866</v>
       </c>
       <c r="F131" s="2" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="G131" s="2" t="n">
-        <v>29875</v>
+        <v>23225</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>275</v>
+        <v>5625</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="132">
@@ -4821,16 +4821,16 @@
         <v>114933</v>
       </c>
       <c r="F132" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>31315</v>
+        <v>25915</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>1715</v>
+        <v>315</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="133">
@@ -4852,16 +4852,16 @@
         <v>125050</v>
       </c>
       <c r="F133" s="2" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="G133" s="2" t="n">
-        <v>32780</v>
+        <v>28830</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>3180</v>
+        <v>3230</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="134">
@@ -4883,16 +4883,16 @@
         <v>135266</v>
       </c>
       <c r="F134" s="2" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G134" s="2" t="n">
-        <v>34295</v>
+        <v>31145</v>
       </c>
       <c r="H134" s="2" t="n">
-        <v>4695</v>
+        <v>5545</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="135">
@@ -4914,16 +4914,16 @@
         <v>145683</v>
       </c>
       <c r="F135" s="2" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G135" s="2" t="n">
-        <v>35910</v>
+        <v>34660</v>
       </c>
       <c r="H135" s="2" t="n">
-        <v>6310</v>
+        <v>1060</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="136">
@@ -4951,7 +4951,7 @@
         <v>37675</v>
       </c>
       <c r="H136" s="2" t="n">
-        <v>8075</v>
+        <v>4075</v>
       </c>
       <c r="I136" s="2" t="n">
         <v>22</v>
@@ -4982,7 +4982,7 @@
         <v>39265</v>
       </c>
       <c r="H137" s="2" t="n">
-        <v>9665</v>
+        <v>5665</v>
       </c>
       <c r="I137" s="2" t="n">
         <v>22</v>
@@ -5013,10 +5013,10 @@
         <v>40680</v>
       </c>
       <c r="H138" s="2" t="n">
-        <v>11080</v>
+        <v>3080</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="139">
@@ -5168,10 +5168,10 @@
         <v>48180</v>
       </c>
       <c r="H143" s="2" t="n">
-        <v>2580</v>
+        <v>10580</v>
       </c>
       <c r="I143" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="144">
@@ -5199,10 +5199,10 @@
         <v>49770</v>
       </c>
       <c r="H144" s="2" t="n">
-        <v>4170</v>
+        <v>12170</v>
       </c>
       <c r="I144" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="145">
@@ -5230,10 +5230,10 @@
         <v>51185</v>
       </c>
       <c r="H145" s="2" t="n">
-        <v>5585</v>
+        <v>13585</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="146">
@@ -5261,10 +5261,10 @@
         <v>52625</v>
       </c>
       <c r="H146" s="2" t="n">
-        <v>7025</v>
+        <v>15025</v>
       </c>
       <c r="I146" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="147">
@@ -5292,10 +5292,10 @@
         <v>54090</v>
       </c>
       <c r="H147" s="2" t="n">
-        <v>8490</v>
+        <v>16490</v>
       </c>
       <c r="I147" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="148">
@@ -5323,10 +5323,10 @@
         <v>55605</v>
       </c>
       <c r="H148" s="2" t="n">
-        <v>10005</v>
+        <v>18005</v>
       </c>
       <c r="I148" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="149">
@@ -5354,10 +5354,10 @@
         <v>57220</v>
       </c>
       <c r="H149" s="2" t="n">
-        <v>11620</v>
+        <v>19620</v>
       </c>
       <c r="I149" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="150">
@@ -5385,10 +5385,10 @@
         <v>58785</v>
       </c>
       <c r="H150" s="2" t="n">
-        <v>13185</v>
+        <v>21185</v>
       </c>
       <c r="I150" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="151">
@@ -5416,10 +5416,10 @@
         <v>60375</v>
       </c>
       <c r="H151" s="2" t="n">
-        <v>14775</v>
+        <v>22775</v>
       </c>
       <c r="I151" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="152">
@@ -5447,10 +5447,10 @@
         <v>61790</v>
       </c>
       <c r="H152" s="2" t="n">
-        <v>16190</v>
+        <v>24190</v>
       </c>
       <c r="I152" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="153">
@@ -6371,16 +6371,16 @@
         <v>3610</v>
       </c>
       <c r="F182" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G182" s="2" t="n">
-        <v>1070</v>
+        <v>500</v>
       </c>
       <c r="H182" s="2" t="n">
-        <v>470</v>
+        <v>500</v>
       </c>
       <c r="I182" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="183">
@@ -6402,16 +6402,16 @@
         <v>6370</v>
       </c>
       <c r="F183" s="2" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="G183" s="2" t="n">
-        <v>1755</v>
+        <v>835</v>
       </c>
       <c r="H183" s="2" t="n">
-        <v>555</v>
+        <v>235</v>
       </c>
       <c r="I183" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184">
@@ -6433,16 +6433,16 @@
         <v>9180</v>
       </c>
       <c r="F184" s="2" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="G184" s="2" t="n">
-        <v>2375</v>
+        <v>1125</v>
       </c>
       <c r="H184" s="2" t="n">
-        <v>575</v>
+        <v>525</v>
       </c>
       <c r="I184" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="185">
@@ -6464,16 +6464,16 @@
         <v>12040</v>
       </c>
       <c r="F185" s="2" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="G185" s="2" t="n">
-        <v>3060</v>
+        <v>1520</v>
       </c>
       <c r="H185" s="2" t="n">
-        <v>660</v>
+        <v>320</v>
       </c>
       <c r="I185" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="186">
@@ -6495,16 +6495,16 @@
         <v>14950</v>
       </c>
       <c r="F186" s="2" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="G186" s="2" t="n">
-        <v>3600</v>
+        <v>1860</v>
       </c>
       <c r="H186" s="2" t="n">
-        <v>1200</v>
+        <v>60</v>
       </c>
       <c r="I186" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="187">
@@ -6526,16 +6526,16 @@
         <v>17960</v>
       </c>
       <c r="F187" s="2" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="G187" s="2" t="n">
-        <v>4450</v>
+        <v>2340</v>
       </c>
       <c r="H187" s="2" t="n">
-        <v>250</v>
+        <v>540</v>
       </c>
       <c r="I187" s="2" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="188">
@@ -6557,16 +6557,16 @@
         <v>21170</v>
       </c>
       <c r="F188" s="2" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G188" s="2" t="n">
-        <v>5480</v>
+        <v>2830</v>
       </c>
       <c r="H188" s="2" t="n">
-        <v>1280</v>
+        <v>430</v>
       </c>
       <c r="I188" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="189">
@@ -6588,16 +6588,16 @@
         <v>25430</v>
       </c>
       <c r="F189" s="2" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="G189" s="2" t="n">
-        <v>7390</v>
+        <v>3630</v>
       </c>
       <c r="H189" s="2" t="n">
-        <v>1390</v>
+        <v>1230</v>
       </c>
       <c r="I189" s="2" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="190">
@@ -6619,16 +6619,16 @@
         <v>28190</v>
       </c>
       <c r="F190" s="2" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G190" s="2" t="n">
-        <v>7655</v>
+        <v>3895</v>
       </c>
       <c r="H190" s="2" t="n">
-        <v>1655</v>
+        <v>1495</v>
       </c>
       <c r="I190" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="191">
@@ -6650,16 +6650,16 @@
         <v>31000</v>
       </c>
       <c r="F191" s="2" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="G191" s="2" t="n">
-        <v>8725</v>
+        <v>4305</v>
       </c>
       <c r="H191" s="2" t="n">
-        <v>2725</v>
+        <v>105</v>
       </c>
       <c r="I191" s="2" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="192">
@@ -6681,16 +6681,16 @@
         <v>33860</v>
       </c>
       <c r="F192" s="2" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="G192" s="2" t="n">
-        <v>9460</v>
+        <v>4620</v>
       </c>
       <c r="H192" s="2" t="n">
-        <v>1660</v>
+        <v>420</v>
       </c>
       <c r="I192" s="2" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="193">
@@ -6712,16 +6712,16 @@
         <v>36770</v>
       </c>
       <c r="F193" s="2" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G193" s="2" t="n">
-        <v>10240</v>
+        <v>4960</v>
       </c>
       <c r="H193" s="2" t="n">
-        <v>640</v>
+        <v>760</v>
       </c>
       <c r="I193" s="2" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="194">
@@ -6743,16 +6743,16 @@
         <v>39780</v>
       </c>
       <c r="F194" s="2" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="G194" s="2" t="n">
-        <v>11090</v>
+        <v>5480</v>
       </c>
       <c r="H194" s="2" t="n">
-        <v>1490</v>
+        <v>1280</v>
       </c>
       <c r="I194" s="2" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="195">
@@ -6774,16 +6774,16 @@
         <v>42990</v>
       </c>
       <c r="F195" s="2" t="n">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="G195" s="2" t="n">
-        <v>12060</v>
+        <v>5970</v>
       </c>
       <c r="H195" s="2" t="n">
-        <v>2460</v>
+        <v>1770</v>
       </c>
       <c r="I195" s="2" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="196">
@@ -6805,16 +6805,16 @@
         <v>47500</v>
       </c>
       <c r="F196" s="2" t="n">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="G196" s="2" t="n">
-        <v>14350</v>
+        <v>6750</v>
       </c>
       <c r="H196" s="2" t="n">
         <v>750</v>
       </c>
       <c r="I196" s="2" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="197">
@@ -6836,16 +6836,16 @@
         <v>50260</v>
       </c>
       <c r="F197" s="2" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="G197" s="2" t="n">
-        <v>15265</v>
+        <v>7165</v>
       </c>
       <c r="H197" s="2" t="n">
-        <v>1665</v>
+        <v>1165</v>
       </c>
       <c r="I197" s="2" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="198">
@@ -6867,16 +6867,16 @@
         <v>53070</v>
       </c>
       <c r="F198" s="2" t="n">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="G198" s="2" t="n">
-        <v>16255</v>
+        <v>7455</v>
       </c>
       <c r="H198" s="2" t="n">
-        <v>2655</v>
+        <v>1455</v>
       </c>
       <c r="I198" s="2" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="199">
@@ -6898,16 +6898,16 @@
         <v>55680</v>
       </c>
       <c r="F199" s="2" t="n">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="G199" s="2" t="n">
-        <v>16520</v>
+        <v>7880</v>
       </c>
       <c r="H199" s="2" t="n">
-        <v>2920</v>
+        <v>1880</v>
       </c>
       <c r="I199" s="2" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="200">
@@ -6929,16 +6929,16 @@
         <v>58590</v>
       </c>
       <c r="F200" s="2" t="n">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G200" s="2" t="n">
-        <v>17610</v>
+        <v>8220</v>
       </c>
       <c r="H200" s="2" t="n">
-        <v>10</v>
+        <v>420</v>
       </c>
       <c r="I200" s="2" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="201">
@@ -6960,16 +6960,16 @@
         <v>61600</v>
       </c>
       <c r="F201" s="2" t="n">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="G201" s="2" t="n">
-        <v>18800</v>
+        <v>8610</v>
       </c>
       <c r="H201" s="2" t="n">
-        <v>1200</v>
+        <v>810</v>
       </c>
       <c r="I201" s="2" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="202">
@@ -6991,16 +6991,16 @@
         <v>64560</v>
       </c>
       <c r="F202" s="2" t="n">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="G202" s="2" t="n">
-        <v>20140</v>
+        <v>9050</v>
       </c>
       <c r="H202" s="2" t="n">
-        <v>2540</v>
+        <v>1250</v>
       </c>
       <c r="I202" s="2" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="203">
@@ -7022,16 +7022,16 @@
         <v>68170</v>
       </c>
       <c r="F203" s="2" t="n">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="G203" s="2" t="n">
-        <v>21580</v>
+        <v>9660</v>
       </c>
       <c r="H203" s="2" t="n">
-        <v>3980</v>
+        <v>60</v>
       </c>
       <c r="I203" s="2" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="204">
@@ -7053,16 +7053,16 @@
         <v>70930</v>
       </c>
       <c r="F204" s="2" t="n">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="G204" s="2" t="n">
-        <v>23095</v>
+        <v>9925</v>
       </c>
       <c r="H204" s="2" t="n">
-        <v>5495</v>
+        <v>325</v>
       </c>
       <c r="I204" s="2" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="205">
@@ -7084,16 +7084,16 @@
         <v>73740</v>
       </c>
       <c r="F205" s="2" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="G205" s="2" t="n">
-        <v>23385</v>
+        <v>10395</v>
       </c>
       <c r="H205" s="2" t="n">
-        <v>5785</v>
+        <v>795</v>
       </c>
       <c r="I205" s="2" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="206">
@@ -7115,16 +7115,16 @@
         <v>76600</v>
       </c>
       <c r="F206" s="2" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="G206" s="2" t="n">
-        <v>23700</v>
+        <v>10710</v>
       </c>
       <c r="H206" s="2" t="n">
-        <v>2100</v>
+        <v>1110</v>
       </c>
       <c r="I206" s="2" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="207">
@@ -7146,16 +7146,16 @@
         <v>79260</v>
       </c>
       <c r="F207" s="2" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="G207" s="2" t="n">
-        <v>23990</v>
+        <v>11000</v>
       </c>
       <c r="H207" s="2" t="n">
-        <v>2390</v>
+        <v>1400</v>
       </c>
       <c r="I207" s="2" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="208">
@@ -7177,16 +7177,16 @@
         <v>82020</v>
       </c>
       <c r="F208" s="2" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="G208" s="2" t="n">
-        <v>24330</v>
+        <v>11530</v>
       </c>
       <c r="H208" s="2" t="n">
-        <v>2730</v>
+        <v>1930</v>
       </c>
       <c r="I208" s="2" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="209">
@@ -7208,16 +7208,16 @@
         <v>85230</v>
       </c>
       <c r="F209" s="2" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="G209" s="2" t="n">
-        <v>24820</v>
+        <v>12020</v>
       </c>
       <c r="H209" s="2" t="n">
-        <v>3220</v>
+        <v>2420</v>
       </c>
       <c r="I209" s="2" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="210">
@@ -7239,16 +7239,16 @@
         <v>88840</v>
       </c>
       <c r="F210" s="2" t="n">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="G210" s="2" t="n">
-        <v>25260</v>
+        <v>12660</v>
       </c>
       <c r="H210" s="2" t="n">
-        <v>3660</v>
+        <v>3060</v>
       </c>
       <c r="I210" s="2" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="211">
@@ -7270,16 +7270,16 @@
         <v>91350</v>
       </c>
       <c r="F211" s="2" t="n">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="G211" s="2" t="n">
-        <v>25475</v>
+        <v>12875</v>
       </c>
       <c r="H211" s="2" t="n">
-        <v>3875</v>
+        <v>3275</v>
       </c>
       <c r="I211" s="2" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="212">
@@ -7301,16 +7301,16 @@
         <v>94160</v>
       </c>
       <c r="F212" s="2" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G212" s="2" t="n">
-        <v>25765</v>
+        <v>13165</v>
       </c>
       <c r="H212" s="2" t="n">
-        <v>4165</v>
+        <v>3565</v>
       </c>
       <c r="I212" s="2" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
     <row r="213">
@@ -7332,16 +7332,16 @@
         <v>96770</v>
       </c>
       <c r="F213" s="2" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G213" s="2" t="n">
-        <v>26030</v>
+        <v>13430</v>
       </c>
       <c r="H213" s="2" t="n">
-        <v>4430</v>
+        <v>3830</v>
       </c>
       <c r="I213" s="2" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
     <row r="214">
@@ -7363,16 +7363,16 @@
         <v>99680</v>
       </c>
       <c r="F214" s="2" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G214" s="2" t="n">
-        <v>26370</v>
+        <v>13770</v>
       </c>
       <c r="H214" s="2" t="n">
-        <v>4770</v>
+        <v>170</v>
       </c>
       <c r="I214" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="215">
@@ -7394,16 +7394,16 @@
         <v>102690</v>
       </c>
       <c r="F215" s="2" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="G215" s="2" t="n">
-        <v>26760</v>
+        <v>14380</v>
       </c>
       <c r="H215" s="2" t="n">
-        <v>5160</v>
+        <v>780</v>
       </c>
       <c r="I215" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="216">
@@ -7425,16 +7425,16 @@
         <v>105900</v>
       </c>
       <c r="F216" s="2" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="G216" s="2" t="n">
-        <v>27250</v>
+        <v>14870</v>
       </c>
       <c r="H216" s="2" t="n">
-        <v>5650</v>
+        <v>1270</v>
       </c>
       <c r="I216" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="217">
@@ -7456,16 +7456,16 @@
         <v>109510</v>
       </c>
       <c r="F217" s="2" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="G217" s="2" t="n">
-        <v>27690</v>
+        <v>15550</v>
       </c>
       <c r="H217" s="2" t="n">
-        <v>6090</v>
+        <v>1950</v>
       </c>
       <c r="I217" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="218">
@@ -7487,16 +7487,16 @@
         <v>112270</v>
       </c>
       <c r="F218" s="2" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="G218" s="2" t="n">
-        <v>27955</v>
+        <v>15815</v>
       </c>
       <c r="H218" s="2" t="n">
-        <v>6355</v>
+        <v>2215</v>
       </c>
       <c r="I218" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="219">
@@ -7518,16 +7518,16 @@
         <v>115080</v>
       </c>
       <c r="F219" s="2" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="G219" s="2" t="n">
-        <v>28245</v>
+        <v>16105</v>
       </c>
       <c r="H219" s="2" t="n">
-        <v>6645</v>
+        <v>2505</v>
       </c>
       <c r="I219" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="220">
@@ -7549,16 +7549,16 @@
         <v>117690</v>
       </c>
       <c r="F220" s="2" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="G220" s="2" t="n">
-        <v>28510</v>
+        <v>16630</v>
       </c>
       <c r="H220" s="2" t="n">
-        <v>6910</v>
+        <v>3030</v>
       </c>
       <c r="I220" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="221">
@@ -7580,16 +7580,16 @@
         <v>120600</v>
       </c>
       <c r="F221" s="2" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="G221" s="2" t="n">
-        <v>28850</v>
+        <v>16970</v>
       </c>
       <c r="H221" s="2" t="n">
-        <v>7250</v>
+        <v>3370</v>
       </c>
       <c r="I221" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="222">
@@ -7611,16 +7611,16 @@
         <v>123610</v>
       </c>
       <c r="F222" s="2" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="G222" s="2" t="n">
-        <v>29240</v>
+        <v>17360</v>
       </c>
       <c r="H222" s="2" t="n">
-        <v>7640</v>
+        <v>3760</v>
       </c>
       <c r="I222" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="223">
@@ -7642,16 +7642,16 @@
         <v>126820</v>
       </c>
       <c r="F223" s="2" t="n">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="G223" s="2" t="n">
-        <v>29730</v>
+        <v>18130</v>
       </c>
       <c r="H223" s="2" t="n">
-        <v>130</v>
+        <v>4530</v>
       </c>
       <c r="I223" s="2" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="224">
@@ -7673,16 +7673,16 @@
         <v>131330</v>
       </c>
       <c r="F224" s="2" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G224" s="2" t="n">
-        <v>30370</v>
+        <v>18770</v>
       </c>
       <c r="H224" s="2" t="n">
-        <v>770</v>
+        <v>5170</v>
       </c>
       <c r="I224" s="2" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="225">
@@ -7704,16 +7704,16 @@
         <v>134090</v>
       </c>
       <c r="F225" s="2" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G225" s="2" t="n">
-        <v>30635</v>
+        <v>19035</v>
       </c>
       <c r="H225" s="2" t="n">
-        <v>1035</v>
+        <v>1435</v>
       </c>
       <c r="I225" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="226">
@@ -7735,16 +7735,16 @@
         <v>136900</v>
       </c>
       <c r="F226" s="2" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G226" s="2" t="n">
-        <v>30925</v>
+        <v>19325</v>
       </c>
       <c r="H226" s="2" t="n">
-        <v>1325</v>
+        <v>1725</v>
       </c>
       <c r="I226" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227">
@@ -7766,16 +7766,16 @@
         <v>139760</v>
       </c>
       <c r="F227" s="2" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="G227" s="2" t="n">
-        <v>31240</v>
+        <v>19940</v>
       </c>
       <c r="H227" s="2" t="n">
-        <v>1640</v>
+        <v>2340</v>
       </c>
       <c r="I227" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="228">
@@ -7797,16 +7797,16 @@
         <v>142670</v>
       </c>
       <c r="F228" s="2" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="G228" s="2" t="n">
-        <v>31580</v>
+        <v>20280</v>
       </c>
       <c r="H228" s="2" t="n">
-        <v>1980</v>
+        <v>2680</v>
       </c>
       <c r="I228" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="229">
@@ -7828,16 +7828,16 @@
         <v>145430</v>
       </c>
       <c r="F229" s="2" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="G229" s="2" t="n">
-        <v>31920</v>
+        <v>20620</v>
       </c>
       <c r="H229" s="2" t="n">
-        <v>2320</v>
+        <v>3020</v>
       </c>
       <c r="I229" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="230">
@@ -7859,16 +7859,16 @@
         <v>148640</v>
       </c>
       <c r="F230" s="2" t="n">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="G230" s="2" t="n">
-        <v>32410</v>
+        <v>21430</v>
       </c>
       <c r="H230" s="2" t="n">
-        <v>2810</v>
+        <v>3830</v>
       </c>
       <c r="I230" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231">
@@ -7890,16 +7890,16 @@
         <v>153150</v>
       </c>
       <c r="F231" s="2" t="n">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="G231" s="2" t="n">
-        <v>33050</v>
+        <v>22070</v>
       </c>
       <c r="H231" s="2" t="n">
-        <v>3450</v>
+        <v>4470</v>
       </c>
       <c r="I231" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="232">
@@ -7921,16 +7921,16 @@
         <v>155910</v>
       </c>
       <c r="F232" s="2" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="G232" s="2" t="n">
-        <v>33315</v>
+        <v>22675</v>
       </c>
       <c r="H232" s="2" t="n">
-        <v>3715</v>
+        <v>5075</v>
       </c>
       <c r="I232" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="233">
@@ -7952,16 +7952,16 @@
         <v>158720</v>
       </c>
       <c r="F233" s="2" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="G233" s="2" t="n">
-        <v>33605</v>
+        <v>22965</v>
       </c>
       <c r="H233" s="2" t="n">
-        <v>4005</v>
+        <v>5365</v>
       </c>
       <c r="I233" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="234">
@@ -7983,16 +7983,16 @@
         <v>161580</v>
       </c>
       <c r="F234" s="2" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="G234" s="2" t="n">
-        <v>33920</v>
+        <v>23280</v>
       </c>
       <c r="H234" s="2" t="n">
-        <v>4320</v>
+        <v>5680</v>
       </c>
       <c r="I234" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="235">
@@ -8014,16 +8014,16 @@
         <v>164490</v>
       </c>
       <c r="F235" s="2" t="n">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="G235" s="2" t="n">
-        <v>34260</v>
+        <v>23980</v>
       </c>
       <c r="H235" s="2" t="n">
-        <v>4660</v>
+        <v>2380</v>
       </c>
       <c r="I235" s="2" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="236">
@@ -8045,16 +8045,16 @@
         <v>167250</v>
       </c>
       <c r="F236" s="2" t="n">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="G236" s="2" t="n">
-        <v>34600</v>
+        <v>24320</v>
       </c>
       <c r="H236" s="2" t="n">
-        <v>5000</v>
+        <v>2720</v>
       </c>
       <c r="I236" s="2" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="237">
@@ -8076,16 +8076,16 @@
         <v>170460</v>
       </c>
       <c r="F237" s="2" t="n">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="G237" s="2" t="n">
-        <v>35090</v>
+        <v>24810</v>
       </c>
       <c r="H237" s="2" t="n">
-        <v>5490</v>
+        <v>3210</v>
       </c>
       <c r="I237" s="2" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="238">
@@ -8107,16 +8107,16 @@
         <v>174970</v>
       </c>
       <c r="F238" s="2" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G238" s="2" t="n">
-        <v>35730</v>
+        <v>25450</v>
       </c>
       <c r="H238" s="2" t="n">
-        <v>6130</v>
+        <v>3850</v>
       </c>
       <c r="I238" s="2" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="239">
@@ -8138,16 +8138,16 @@
         <v>177730</v>
       </c>
       <c r="F239" s="2" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G239" s="2" t="n">
-        <v>35995</v>
+        <v>25715</v>
       </c>
       <c r="H239" s="2" t="n">
-        <v>6395</v>
+        <v>4115</v>
       </c>
       <c r="I239" s="2" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="240">
@@ -8169,16 +8169,16 @@
         <v>180540</v>
       </c>
       <c r="F240" s="2" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="G240" s="2" t="n">
-        <v>36285</v>
+        <v>26385</v>
       </c>
       <c r="H240" s="2" t="n">
-        <v>6685</v>
+        <v>4785</v>
       </c>
       <c r="I240" s="2" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="241">
@@ -8200,16 +8200,16 @@
         <v>183400</v>
       </c>
       <c r="F241" s="2" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="G241" s="2" t="n">
-        <v>36600</v>
+        <v>26700</v>
       </c>
       <c r="H241" s="2" t="n">
-        <v>7000</v>
+        <v>5100</v>
       </c>
       <c r="I241" s="2" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>